<commit_message>
Added more airbrakes sim graphs
</commit_message>
<xml_diff>
--- a/night_fury_3-22-26_airbrakes_input.xlsx
+++ b/night_fury_3-22-26_airbrakes_input.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brady\repos\UCI-Rocket-Project-Solids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8736C5B6-9041-40CA-9935-4735936785E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED53E910-6A92-476A-980B-284E438E3EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>altitude</t>
   </si>
@@ -55,6 +66,9 @@
   </si>
   <si>
     <t>pressure</t>
+  </si>
+  <si>
+    <t>temperature</t>
   </si>
 </sst>
 </file>
@@ -372,10 +386,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -406,8 +420,11 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>648890</v>
       </c>
@@ -438,8 +455,11 @@
       <c r="J2">
         <v>937.31299999999999</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2">
+        <v>44.21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>649890</v>
       </c>
@@ -470,8 +490,11 @@
       <c r="J3">
         <v>937.33699999999999</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <v>44.21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>650890</v>
       </c>
@@ -502,8 +525,11 @@
       <c r="J4">
         <v>937.31299999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <v>44.22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>651889</v>
       </c>
@@ -534,8 +560,11 @@
       <c r="J5">
         <v>937.31399999999996</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5">
+        <v>44.22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>652889</v>
       </c>
@@ -566,8 +595,11 @@
       <c r="J6">
         <v>934.53700000000003</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6">
+        <v>44.14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>653889</v>
       </c>
@@ -598,8 +630,11 @@
       <c r="J7">
         <v>921.94100000000003</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <v>43.94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>654889</v>
       </c>
@@ -630,8 +665,11 @@
       <c r="J8">
         <v>899.798</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8">
+        <v>44.16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>655889</v>
       </c>
@@ -662,8 +700,11 @@
       <c r="J9">
         <v>875.28200000000004</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9">
+        <v>44.21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>656889</v>
       </c>
@@ -694,8 +735,11 @@
       <c r="J10">
         <v>852.04499999999996</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <v>44.18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>657890</v>
       </c>
@@ -726,8 +770,11 @@
       <c r="J11">
         <v>830.47</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11">
+        <v>44.15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>658889</v>
       </c>
@@ -758,8 +805,11 @@
       <c r="J12">
         <v>810.97900000000004</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12">
+        <v>44.03</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>659889</v>
       </c>
@@ -790,8 +840,11 @@
       <c r="J13">
         <v>793.303</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <v>43.83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>660890</v>
       </c>
@@ -822,8 +875,11 @@
       <c r="J14">
         <v>777.47299999999996</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <v>43.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>661890</v>
       </c>
@@ -854,8 +910,11 @@
       <c r="J15">
         <v>762.97400000000005</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>662890</v>
       </c>
@@ -886,8 +945,11 @@
       <c r="J16">
         <v>749.82100000000003</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <v>43.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>663889</v>
       </c>
@@ -918,8 +980,11 @@
       <c r="J17">
         <v>738.17</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <v>43.07</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>664890</v>
       </c>
@@ -950,8 +1015,11 @@
       <c r="J18">
         <v>727.49</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <v>42.93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>665889</v>
       </c>
@@ -982,8 +1050,11 @@
       <c r="J19">
         <v>717.95799999999997</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <v>42.79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>666890</v>
       </c>
@@ -1014,8 +1085,11 @@
       <c r="J20">
         <v>709.52700000000004</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <v>42.69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>667890</v>
       </c>
@@ -1046,8 +1120,11 @@
       <c r="J21">
         <v>702.14</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <v>42.59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>668889</v>
       </c>
@@ -1078,8 +1155,11 @@
       <c r="J22">
         <v>695.68700000000001</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <v>42.53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>669889</v>
       </c>
@@ -1110,8 +1190,11 @@
       <c r="J23">
         <v>690.12599999999998</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23">
+        <v>42.47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>670889</v>
       </c>
@@ -1142,8 +1225,11 @@
       <c r="J24">
         <v>685.46299999999997</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24">
+        <v>42.35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>671889</v>
       </c>
@@ -1174,8 +1260,11 @@
       <c r="J25">
         <v>681.75900000000001</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25">
+        <v>42.34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>672890</v>
       </c>
@@ -1206,8 +1295,11 @@
       <c r="J26">
         <v>678.85199999999998</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26">
+        <v>42.29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>673890</v>
       </c>
@@ -1238,8 +1330,11 @@
       <c r="J27">
         <v>676.72500000000002</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27">
+        <v>42.37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>674890</v>
       </c>
@@ -1270,8 +1365,11 @@
       <c r="J28">
         <v>675.45799999999997</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28">
+        <v>42.38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>675890</v>
       </c>
@@ -1302,8 +1400,11 @@
       <c r="J29">
         <v>675.02300000000002</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29">
+        <v>42.33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>676890</v>
       </c>
@@ -1334,8 +1435,11 @@
       <c r="J30">
         <v>675.32399999999996</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30">
+        <v>42.24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>677890</v>
       </c>
@@ -1365,6 +1469,9 @@
       </c>
       <c r="J31">
         <v>676.19899999999996</v>
+      </c>
+      <c r="K31">
+        <v>42.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Messing with using old data
</commit_message>
<xml_diff>
--- a/night_fury_3-22-26_airbrakes_input.xlsx
+++ b/night_fury_3-22-26_airbrakes_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brady\repos\UCI-Rocket-Project-Solids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8C374C-9F1A-48EE-AE77-6B9B21EC218D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4075780C-E1DC-4FBF-ABD7-3BC06A58AC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>altitude</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>alt_fused</t>
+  </si>
+  <si>
+    <t>accel_world_z</t>
   </si>
 </sst>
 </file>
@@ -389,10 +392,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -429,8 +432,11 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>648890</v>
       </c>
@@ -467,8 +473,11 @@
       <c r="L2">
         <v>2.0419999999999998</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M2">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>649890</v>
       </c>
@@ -505,8 +514,11 @@
       <c r="L3">
         <v>1.931</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>650890</v>
       </c>
@@ -543,8 +555,11 @@
       <c r="L4">
         <v>1.9490000000000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4">
+        <v>-6.3E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>651889</v>
       </c>
@@ -581,8 +596,11 @@
       <c r="L5">
         <v>2.0350000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5">
+        <v>2.4420000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>652889</v>
       </c>
@@ -619,8 +637,11 @@
       <c r="L6">
         <v>15.353</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6">
+        <v>28.827000000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>653889</v>
       </c>
@@ -657,8 +678,11 @@
       <c r="L7">
         <v>103.90300000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M7">
+        <v>28.271999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>654889</v>
       </c>
@@ -695,8 +719,11 @@
       <c r="L8">
         <v>297.34800000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M8">
+        <v>24.204000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>655889</v>
       </c>
@@ -733,8 +760,11 @@
       <c r="L9">
         <v>541.58900000000006</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M9">
+        <v>-5.8150000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>656889</v>
       </c>
@@ -771,8 +801,11 @@
       <c r="L10">
         <v>778.43799999999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M10">
+        <v>-14.632999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>657890</v>
       </c>
@@ -809,8 +842,11 @@
       <c r="L11">
         <v>996.62900000000002</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M11">
+        <v>-16.673999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>658889</v>
       </c>
@@ -847,8 +883,11 @@
       <c r="L12">
         <v>1193.211</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M12">
+        <v>-16.273</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>659889</v>
       </c>
@@ -885,8 +924,11 @@
       <c r="L13">
         <v>1372.0909999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M13">
+        <v>-15.382999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>660890</v>
       </c>
@@ -923,8 +965,11 @@
       <c r="L14">
         <v>1535.893</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M14">
+        <v>-14.56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>661890</v>
       </c>
@@ -961,8 +1006,11 @@
       <c r="L15">
         <v>1686.221</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M15">
+        <v>-13.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>662890</v>
       </c>
@@ -999,8 +1047,11 @@
       <c r="L16">
         <v>1824.06</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M16">
+        <v>-12.539</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>663889</v>
       </c>
@@ -1037,8 +1088,11 @@
       <c r="L17">
         <v>1949.3150000000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M17">
+        <v>-12.507</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>664890</v>
       </c>
@@ -1075,8 +1129,11 @@
       <c r="L18">
         <v>2064.2339999999999</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M18">
+        <v>-12.051</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>665889</v>
       </c>
@@ -1113,8 +1170,11 @@
       <c r="L19">
         <v>2168.299</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M19">
+        <v>-11.385</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>666890</v>
       </c>
@@ -1151,8 +1211,11 @@
       <c r="L20">
         <v>2261.5070000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M20">
+        <v>-11.362</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>667890</v>
       </c>
@@ -1189,8 +1252,11 @@
       <c r="L21">
         <v>2343.922</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M21">
+        <v>-10.743</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>668889</v>
       </c>
@@ -1227,8 +1293,11 @@
       <c r="L22">
         <v>2416.471</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M22">
+        <v>-10.708</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>669889</v>
       </c>
@@ -1265,8 +1334,11 @@
       <c r="L23">
         <v>2478.7820000000002</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M23">
+        <v>-10.237</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>670889</v>
       </c>
@@ -1303,8 +1375,11 @@
       <c r="L24">
         <v>2531.625</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M24">
+        <v>-10.172000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>671889</v>
       </c>
@@ -1341,8 +1416,11 @@
       <c r="L25">
         <v>2574.5039999999999</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M25">
+        <v>-10.321</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>672890</v>
       </c>
@@ -1379,8 +1457,11 @@
       <c r="L26">
         <v>2607.8420000000001</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M26">
+        <v>-9.8989999999999991</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>673890</v>
       </c>
@@ -1417,8 +1498,11 @@
       <c r="L27">
         <v>2632.0520000000001</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M27">
+        <v>-9.7850000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>674890</v>
       </c>
@@ -1455,8 +1539,11 @@
       <c r="L28">
         <v>2646.6390000000001</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M28">
+        <v>-9.7140000000000004</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>675890</v>
       </c>
@@ -1493,8 +1580,11 @@
       <c r="L29">
         <v>2652.127</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M29">
+        <v>-9.7850000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>676890</v>
       </c>
@@ -1531,8 +1621,11 @@
       <c r="L30">
         <v>2648.1129999999998</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M30">
+        <v>-9.7409999999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>677890</v>
       </c>
@@ -1568,6 +1661,9 @@
       </c>
       <c r="L31">
         <v>2635.357</v>
+      </c>
+      <c r="M31">
+        <v>-8.7129999999999992</v>
       </c>
     </row>
   </sheetData>

</xml_diff>